<commit_message>
updated .svg plot notation
</commit_message>
<xml_diff>
--- a/NfL-iPLA_imprecision/Analytical_Precision_Pathology_convention.xlsx
+++ b/NfL-iPLA_imprecision/Analytical_Precision_Pathology_convention.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wehieduau-my.sharepoint.com/personal/smith_j_wehi_edu_au/Documents/Documents/CFHAC_ProxiPal/ProxiPal/user_documents/NfL-PLA Development Paper/NfL-PLA Development Paper Figure Data/GitHub/NfL-iPLA-paper/NfL-iPLA_imprecision/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="266" documentId="8_{5AF014E8-1630-426D-9D80-6B5DABD0E8D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A21CA654-17F2-4D36-B687-06964E54804C}"/>
+  <xr:revisionPtr revIDLastSave="268" documentId="8_{5AF014E8-1630-426D-9D80-6B5DABD0E8D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA8A7C96-6458-4CCE-B305-9F5696E0E116}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="34140" windowHeight="19245" activeTab="1" xr2:uid="{C276D241-3180-455D-B1F9-2AC79E2509AD}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{C276D241-3180-455D-B1F9-2AC79E2509AD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -784,34 +784,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CDE6C01-6100-46C3-80E9-918D22313C58}">
   <dimension ref="B2:AF81"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="13.28515625" customWidth="1"/>
-    <col min="3" max="3" width="13.140625" customWidth="1"/>
-    <col min="4" max="4" width="10.7109375" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" customWidth="1"/>
-    <col min="6" max="11" width="12.5703125" customWidth="1"/>
+    <col min="2" max="2" width="13.26953125" customWidth="1"/>
+    <col min="3" max="3" width="13.1796875" customWidth="1"/>
+    <col min="4" max="4" width="10.7265625" customWidth="1"/>
+    <col min="5" max="5" width="11.7265625" customWidth="1"/>
+    <col min="6" max="11" width="12.54296875" customWidth="1"/>
     <col min="13" max="13" width="12" customWidth="1"/>
-    <col min="14" max="14" width="15.28515625" customWidth="1"/>
-    <col min="15" max="15" width="13.85546875" customWidth="1"/>
-    <col min="16" max="16" width="15.85546875" customWidth="1"/>
-    <col min="19" max="19" width="12.85546875" customWidth="1"/>
-    <col min="20" max="20" width="12.5703125" customWidth="1"/>
-    <col min="21" max="21" width="13.85546875" customWidth="1"/>
-    <col min="22" max="22" width="11.140625" customWidth="1"/>
+    <col min="14" max="14" width="15.26953125" customWidth="1"/>
+    <col min="15" max="15" width="13.81640625" customWidth="1"/>
+    <col min="16" max="16" width="15.81640625" customWidth="1"/>
+    <col min="19" max="19" width="12.81640625" customWidth="1"/>
+    <col min="20" max="20" width="12.54296875" customWidth="1"/>
+    <col min="21" max="21" width="13.81640625" customWidth="1"/>
+    <col min="22" max="22" width="11.1796875" customWidth="1"/>
     <col min="23" max="24" width="11" customWidth="1"/>
-    <col min="27" max="27" width="12.140625" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" customWidth="1"/>
-    <col min="29" max="29" width="12.7109375" customWidth="1"/>
-    <col min="30" max="30" width="10.5703125" customWidth="1"/>
+    <col min="27" max="27" width="12.1796875" customWidth="1"/>
+    <col min="28" max="28" width="10.7265625" customWidth="1"/>
+    <col min="29" max="29" width="12.7265625" customWidth="1"/>
+    <col min="30" max="30" width="10.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B2" s="42" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B3" s="22"/>
       <c r="C3" s="17"/>
       <c r="D3" s="17"/>
@@ -850,7 +850,7 @@
       <c r="AE3" s="28"/>
       <c r="AF3" s="39"/>
     </row>
-    <row r="4" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B4" s="13" t="s">
         <v>1</v>
       </c>
@@ -937,7 +937,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B5" s="6">
         <v>1</v>
       </c>
@@ -992,7 +992,7 @@
       <c r="AE5" s="28"/>
       <c r="AF5" s="39"/>
     </row>
-    <row r="6" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B6" s="11">
         <v>1</v>
       </c>
@@ -1047,7 +1047,7 @@
       <c r="AE6" s="2"/>
       <c r="AF6" s="40"/>
     </row>
-    <row r="7" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B7" s="11">
         <v>1</v>
       </c>
@@ -1102,7 +1102,7 @@
       <c r="AE7" s="2"/>
       <c r="AF7" s="40"/>
     </row>
-    <row r="8" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B8" s="11">
         <v>1</v>
       </c>
@@ -1157,7 +1157,7 @@
       <c r="AE8" s="2"/>
       <c r="AF8" s="40"/>
     </row>
-    <row r="9" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B9" s="11">
         <v>1</v>
       </c>
@@ -1212,7 +1212,7 @@
       <c r="AE9" s="2"/>
       <c r="AF9" s="40"/>
     </row>
-    <row r="10" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B10" s="11">
         <v>1</v>
       </c>
@@ -1267,7 +1267,7 @@
       <c r="AE10" s="2"/>
       <c r="AF10" s="40"/>
     </row>
-    <row r="11" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B11" s="11">
         <v>1</v>
       </c>
@@ -1322,7 +1322,7 @@
       <c r="AE11" s="2"/>
       <c r="AF11" s="40"/>
     </row>
-    <row r="12" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B12" s="11">
         <v>1</v>
       </c>
@@ -1377,7 +1377,7 @@
       <c r="AE12" s="2"/>
       <c r="AF12" s="40"/>
     </row>
-    <row r="13" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B13" s="11">
         <v>1</v>
       </c>
@@ -1432,7 +1432,7 @@
       <c r="AE13" s="2"/>
       <c r="AF13" s="40"/>
     </row>
-    <row r="14" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B14" s="11">
         <v>1</v>
       </c>
@@ -1532,7 +1532,7 @@
         <v>15.792860585090285</v>
       </c>
     </row>
-    <row r="15" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B15" s="6">
         <v>2</v>
       </c>
@@ -1587,7 +1587,7 @@
       <c r="AE15" s="28"/>
       <c r="AF15" s="39"/>
     </row>
-    <row r="16" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B16" s="11">
         <v>2</v>
       </c>
@@ -1642,7 +1642,7 @@
       <c r="AE16" s="2"/>
       <c r="AF16" s="40"/>
     </row>
-    <row r="17" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B17" s="11">
         <v>2</v>
       </c>
@@ -1697,7 +1697,7 @@
       <c r="AE17" s="2"/>
       <c r="AF17" s="40"/>
     </row>
-    <row r="18" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B18" s="11">
         <v>2</v>
       </c>
@@ -1752,7 +1752,7 @@
       <c r="AE18" s="2"/>
       <c r="AF18" s="40"/>
     </row>
-    <row r="19" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B19" s="11">
         <v>2</v>
       </c>
@@ -1807,7 +1807,7 @@
       <c r="AE19" s="2"/>
       <c r="AF19" s="40"/>
     </row>
-    <row r="20" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B20" s="11">
         <v>2</v>
       </c>
@@ -1862,7 +1862,7 @@
       <c r="AE20" s="2"/>
       <c r="AF20" s="40"/>
     </row>
-    <row r="21" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B21" s="11">
         <v>2</v>
       </c>
@@ -1917,7 +1917,7 @@
       <c r="AE21" s="2"/>
       <c r="AF21" s="40"/>
     </row>
-    <row r="22" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B22" s="11">
         <v>2</v>
       </c>
@@ -1972,7 +1972,7 @@
       <c r="AE22" s="2"/>
       <c r="AF22" s="40"/>
     </row>
-    <row r="23" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B23" s="13">
         <v>2</v>
       </c>
@@ -2039,7 +2039,7 @@
       <c r="AE23" s="2"/>
       <c r="AF23" s="40"/>
     </row>
-    <row r="24" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B24" s="6">
         <v>3</v>
       </c>
@@ -2127,7 +2127,7 @@
         <v>16.341485802915539</v>
       </c>
     </row>
-    <row r="25" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B25" s="11">
         <v>3</v>
       </c>
@@ -2184,7 +2184,7 @@
       <c r="AE25" s="28"/>
       <c r="AF25" s="39"/>
     </row>
-    <row r="26" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B26" s="11">
         <v>3</v>
       </c>
@@ -2241,7 +2241,7 @@
       <c r="AE26" s="2"/>
       <c r="AF26" s="40"/>
     </row>
-    <row r="27" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B27" s="11">
         <v>3</v>
       </c>
@@ -2298,7 +2298,7 @@
       <c r="AE27" s="2"/>
       <c r="AF27" s="40"/>
     </row>
-    <row r="28" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B28" s="11">
         <v>3</v>
       </c>
@@ -2355,7 +2355,7 @@
       <c r="AE28" s="2"/>
       <c r="AF28" s="40"/>
     </row>
-    <row r="29" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B29" s="11">
         <v>3</v>
       </c>
@@ -2412,7 +2412,7 @@
       <c r="AE29" s="2"/>
       <c r="AF29" s="40"/>
     </row>
-    <row r="30" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B30" s="11">
         <v>3</v>
       </c>
@@ -2469,7 +2469,7 @@
       <c r="AE30" s="2"/>
       <c r="AF30" s="40"/>
     </row>
-    <row r="31" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B31" s="11">
         <v>3</v>
       </c>
@@ -2526,7 +2526,7 @@
       <c r="AE31" s="2"/>
       <c r="AF31" s="40"/>
     </row>
-    <row r="32" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B32" s="11">
         <v>3</v>
       </c>
@@ -2592,7 +2592,7 @@
         <v>11.995541941166838</v>
       </c>
     </row>
-    <row r="33" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B33" s="13">
         <v>3</v>
       </c>
@@ -2661,7 +2661,7 @@
       <c r="AE33" s="28"/>
       <c r="AF33" s="39"/>
     </row>
-    <row r="34" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B34" s="11">
         <v>4</v>
       </c>
@@ -2740,7 +2740,7 @@
       <c r="AE34" s="2"/>
       <c r="AF34" s="40"/>
     </row>
-    <row r="35" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B35" s="11">
         <v>4</v>
       </c>
@@ -2795,7 +2795,7 @@
       <c r="AE35" s="2"/>
       <c r="AF35" s="40"/>
     </row>
-    <row r="36" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B36" s="11">
         <v>4</v>
       </c>
@@ -2859,7 +2859,7 @@
         <v>13.592134752219362</v>
       </c>
     </row>
-    <row r="37" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B37" s="11">
         <v>4</v>
       </c>
@@ -2916,7 +2916,7 @@
         <v>14.430505770348006</v>
       </c>
     </row>
-    <row r="38" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B38" s="11">
         <v>4</v>
       </c>
@@ -2976,7 +2976,7 @@
         <v>11.780184646827356</v>
       </c>
     </row>
-    <row r="39" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B39" s="13">
         <v>4</v>
       </c>
@@ -3048,7 +3048,7 @@
         <v>18.399887376710556</v>
       </c>
     </row>
-    <row r="40" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B40" s="24" t="s">
         <v>11</v>
       </c>
@@ -3114,7 +3114,7 @@
         <v>11.248660267146384</v>
       </c>
     </row>
-    <row r="41" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B41" t="s">
         <v>12</v>
       </c>
@@ -3157,7 +3157,7 @@
         <v>10.704819498388627</v>
       </c>
     </row>
-    <row r="42" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B42" t="s">
         <v>13</v>
       </c>
@@ -3208,7 +3208,7 @@
       </c>
       <c r="AB42" s="3"/>
     </row>
-    <row r="43" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:32" x14ac:dyDescent="0.35">
       <c r="J43" t="s">
         <v>13</v>
       </c>
@@ -3242,7 +3242,7 @@
         <v>12.890736472214234</v>
       </c>
     </row>
-    <row r="47" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B47" s="22"/>
       <c r="C47" s="17"/>
       <c r="D47" s="17"/>
@@ -3271,7 +3271,7 @@
       <c r="W47" s="17"/>
       <c r="X47" s="18"/>
     </row>
-    <row r="48" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B48" s="13" t="s">
         <v>1</v>
       </c>
@@ -3336,7 +3336,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="49" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B49" s="6">
         <v>1</v>
       </c>
@@ -3377,7 +3377,7 @@
       <c r="W49" s="28"/>
       <c r="X49" s="39"/>
     </row>
-    <row r="50" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B50" s="11">
         <v>1</v>
       </c>
@@ -3418,7 +3418,7 @@
       <c r="W50" s="2"/>
       <c r="X50" s="40"/>
     </row>
-    <row r="51" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B51" s="11">
         <v>1</v>
       </c>
@@ -3459,7 +3459,7 @@
       <c r="W51" s="2"/>
       <c r="X51" s="40"/>
     </row>
-    <row r="52" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B52" s="11">
         <v>1</v>
       </c>
@@ -3500,7 +3500,7 @@
       <c r="W52" s="2"/>
       <c r="X52" s="40"/>
     </row>
-    <row r="53" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B53" s="11">
         <v>1</v>
       </c>
@@ -3541,7 +3541,7 @@
       <c r="W53" s="2"/>
       <c r="X53" s="40"/>
     </row>
-    <row r="54" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B54" s="11">
         <v>1</v>
       </c>
@@ -3582,7 +3582,7 @@
       <c r="W54" s="2"/>
       <c r="X54" s="40"/>
     </row>
-    <row r="55" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B55" s="11">
         <v>1</v>
       </c>
@@ -3623,7 +3623,7 @@
       <c r="W55" s="2"/>
       <c r="X55" s="40"/>
     </row>
-    <row r="56" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B56" s="11">
         <v>1</v>
       </c>
@@ -3664,7 +3664,7 @@
       <c r="W56" s="2"/>
       <c r="X56" s="40"/>
     </row>
-    <row r="57" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B57" s="11">
         <v>1</v>
       </c>
@@ -3705,7 +3705,7 @@
       <c r="W57" s="2"/>
       <c r="X57" s="40"/>
     </row>
-    <row r="58" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B58" s="13">
         <v>1</v>
       </c>
@@ -3782,7 +3782,7 @@
         <v>12.467552636726225</v>
       </c>
     </row>
-    <row r="59" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B59" s="6">
         <v>2</v>
       </c>
@@ -3823,7 +3823,7 @@
       <c r="W59" s="28"/>
       <c r="X59" s="39"/>
     </row>
-    <row r="60" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B60" s="11">
         <v>2</v>
       </c>
@@ -3864,7 +3864,7 @@
       <c r="W60" s="2"/>
       <c r="X60" s="40"/>
     </row>
-    <row r="61" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B61" s="11">
         <v>2</v>
       </c>
@@ -3905,7 +3905,7 @@
       <c r="W61" s="2"/>
       <c r="X61" s="40"/>
     </row>
-    <row r="62" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B62" s="11">
         <v>2</v>
       </c>
@@ -3946,7 +3946,7 @@
       <c r="W62" s="2"/>
       <c r="X62" s="40"/>
     </row>
-    <row r="63" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B63" s="11">
         <v>2</v>
       </c>
@@ -3987,7 +3987,7 @@
       <c r="W63" s="2"/>
       <c r="X63" s="40"/>
     </row>
-    <row r="64" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B64" s="11">
         <v>2</v>
       </c>
@@ -4028,7 +4028,7 @@
       <c r="W64" s="2"/>
       <c r="X64" s="40"/>
     </row>
-    <row r="65" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B65" s="11">
         <v>2</v>
       </c>
@@ -4069,7 +4069,7 @@
       <c r="W65" s="2"/>
       <c r="X65" s="40"/>
     </row>
-    <row r="66" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B66" s="11">
         <v>2</v>
       </c>
@@ -4110,7 +4110,7 @@
       <c r="W66" s="2"/>
       <c r="X66" s="40"/>
     </row>
-    <row r="67" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B67" s="11">
         <v>2</v>
       </c>
@@ -4151,7 +4151,7 @@
       <c r="W67" s="2"/>
       <c r="X67" s="40"/>
     </row>
-    <row r="68" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B68" s="13">
         <v>2</v>
       </c>
@@ -4228,7 +4228,7 @@
         <v>14.19505253988679</v>
       </c>
     </row>
-    <row r="69" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B69" s="6">
         <v>3</v>
       </c>
@@ -4269,7 +4269,7 @@
       <c r="W69" s="28"/>
       <c r="X69" s="39"/>
     </row>
-    <row r="70" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B70" s="11">
         <v>3</v>
       </c>
@@ -4310,7 +4310,7 @@
       <c r="W70" s="2"/>
       <c r="X70" s="40"/>
     </row>
-    <row r="71" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B71" s="11">
         <v>3</v>
       </c>
@@ -4351,7 +4351,7 @@
       <c r="W71" s="2"/>
       <c r="X71" s="40"/>
     </row>
-    <row r="72" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B72" s="11">
         <v>3</v>
       </c>
@@ -4392,7 +4392,7 @@
       <c r="W72" s="2"/>
       <c r="X72" s="40"/>
     </row>
-    <row r="73" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B73" s="11">
         <v>3</v>
       </c>
@@ -4433,7 +4433,7 @@
       <c r="W73" s="2"/>
       <c r="X73" s="40"/>
     </row>
-    <row r="74" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B74" s="11">
         <v>3</v>
       </c>
@@ -4474,7 +4474,7 @@
       <c r="W74" s="2"/>
       <c r="X74" s="40"/>
     </row>
-    <row r="75" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B75" s="11">
         <v>3</v>
       </c>
@@ -4515,7 +4515,7 @@
       <c r="W75" s="2"/>
       <c r="X75" s="40"/>
     </row>
-    <row r="76" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B76" s="11">
         <v>3</v>
       </c>
@@ -4556,7 +4556,7 @@
       <c r="W76" s="2"/>
       <c r="X76" s="40"/>
     </row>
-    <row r="77" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B77" s="11">
         <v>3</v>
       </c>
@@ -4597,7 +4597,7 @@
       <c r="W77" s="2"/>
       <c r="X77" s="40"/>
     </row>
-    <row r="78" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B78" s="13">
         <v>3</v>
       </c>
@@ -4674,7 +4674,7 @@
         <v>13.739374608186964</v>
       </c>
     </row>
-    <row r="79" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B79" s="24" t="s">
         <v>11</v>
       </c>
@@ -4715,7 +4715,7 @@
         <v>13.467326594933326</v>
       </c>
     </row>
-    <row r="80" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B80" t="s">
         <v>12</v>
       </c>
@@ -4774,7 +4774,7 @@
         <v>3.7875326427181033</v>
       </c>
     </row>
-    <row r="81" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B81" t="s">
         <v>13</v>
       </c>
@@ -4842,34 +4842,34 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB3581E6-ADC9-4047-A6F2-5BD73521374E}">
   <dimension ref="B2:AF81"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="13.28515625" customWidth="1"/>
-    <col min="3" max="3" width="13.140625" customWidth="1"/>
-    <col min="4" max="4" width="10.7109375" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" customWidth="1"/>
-    <col min="6" max="11" width="12.5703125" customWidth="1"/>
+    <col min="2" max="2" width="13.26953125" customWidth="1"/>
+    <col min="3" max="3" width="13.1796875" customWidth="1"/>
+    <col min="4" max="4" width="10.7265625" customWidth="1"/>
+    <col min="5" max="5" width="11.7265625" customWidth="1"/>
+    <col min="6" max="11" width="12.54296875" customWidth="1"/>
     <col min="13" max="13" width="12" customWidth="1"/>
-    <col min="14" max="14" width="15.28515625" customWidth="1"/>
-    <col min="15" max="15" width="13.85546875" customWidth="1"/>
-    <col min="16" max="16" width="15.85546875" customWidth="1"/>
-    <col min="19" max="19" width="12.85546875" customWidth="1"/>
-    <col min="20" max="20" width="12.5703125" customWidth="1"/>
-    <col min="21" max="21" width="13.85546875" customWidth="1"/>
-    <col min="22" max="22" width="11.140625" customWidth="1"/>
+    <col min="14" max="14" width="15.26953125" customWidth="1"/>
+    <col min="15" max="15" width="13.81640625" customWidth="1"/>
+    <col min="16" max="16" width="15.81640625" customWidth="1"/>
+    <col min="19" max="19" width="12.81640625" customWidth="1"/>
+    <col min="20" max="20" width="12.54296875" customWidth="1"/>
+    <col min="21" max="21" width="13.81640625" customWidth="1"/>
+    <col min="22" max="22" width="11.1796875" customWidth="1"/>
     <col min="23" max="24" width="11" customWidth="1"/>
-    <col min="27" max="27" width="12.140625" customWidth="1"/>
-    <col min="28" max="28" width="10.7109375" customWidth="1"/>
-    <col min="29" max="29" width="12.7109375" customWidth="1"/>
-    <col min="30" max="30" width="10.5703125" customWidth="1"/>
+    <col min="27" max="27" width="12.1796875" customWidth="1"/>
+    <col min="28" max="28" width="10.7265625" customWidth="1"/>
+    <col min="29" max="29" width="12.7265625" customWidth="1"/>
+    <col min="30" max="30" width="10.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B2" s="42" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B3" s="22"/>
       <c r="C3" s="17"/>
       <c r="D3" s="17"/>
@@ -4908,7 +4908,7 @@
       <c r="AE3" s="28"/>
       <c r="AF3" s="39"/>
     </row>
-    <row r="4" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B4" s="13" t="s">
         <v>1</v>
       </c>
@@ -4995,7 +4995,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B5" s="6">
         <v>1</v>
       </c>
@@ -5050,7 +5050,7 @@
       <c r="AE5" s="28"/>
       <c r="AF5" s="39"/>
     </row>
-    <row r="6" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B6" s="11">
         <v>1</v>
       </c>
@@ -5105,7 +5105,7 @@
       <c r="AE6" s="2"/>
       <c r="AF6" s="40"/>
     </row>
-    <row r="7" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B7" s="11">
         <v>1</v>
       </c>
@@ -5160,7 +5160,7 @@
       <c r="AE7" s="2"/>
       <c r="AF7" s="40"/>
     </row>
-    <row r="8" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B8" s="11">
         <v>1</v>
       </c>
@@ -5215,7 +5215,7 @@
       <c r="AE8" s="2"/>
       <c r="AF8" s="40"/>
     </row>
-    <row r="9" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B9" s="11">
         <v>1</v>
       </c>
@@ -5270,7 +5270,7 @@
       <c r="AE9" s="2"/>
       <c r="AF9" s="40"/>
     </row>
-    <row r="10" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B10" s="11">
         <v>1</v>
       </c>
@@ -5325,7 +5325,7 @@
       <c r="AE10" s="2"/>
       <c r="AF10" s="40"/>
     </row>
-    <row r="11" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B11" s="11">
         <v>1</v>
       </c>
@@ -5380,7 +5380,7 @@
       <c r="AE11" s="2"/>
       <c r="AF11" s="40"/>
     </row>
-    <row r="12" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B12" s="11">
         <v>1</v>
       </c>
@@ -5435,7 +5435,7 @@
       <c r="AE12" s="2"/>
       <c r="AF12" s="40"/>
     </row>
-    <row r="13" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B13" s="11">
         <v>1</v>
       </c>
@@ -5490,7 +5490,7 @@
       <c r="AE13" s="2"/>
       <c r="AF13" s="40"/>
     </row>
-    <row r="14" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B14" s="11">
         <v>1</v>
       </c>
@@ -5590,7 +5590,7 @@
         <v>15.792860585090285</v>
       </c>
     </row>
-    <row r="15" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B15" s="6">
         <v>2</v>
       </c>
@@ -5645,7 +5645,7 @@
       <c r="AE15" s="28"/>
       <c r="AF15" s="39"/>
     </row>
-    <row r="16" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B16" s="11">
         <v>2</v>
       </c>
@@ -5700,7 +5700,7 @@
       <c r="AE16" s="2"/>
       <c r="AF16" s="40"/>
     </row>
-    <row r="17" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B17" s="11">
         <v>2</v>
       </c>
@@ -5755,7 +5755,7 @@
       <c r="AE17" s="2"/>
       <c r="AF17" s="40"/>
     </row>
-    <row r="18" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B18" s="11">
         <v>2</v>
       </c>
@@ -5810,7 +5810,7 @@
       <c r="AE18" s="2"/>
       <c r="AF18" s="40"/>
     </row>
-    <row r="19" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B19" s="11">
         <v>2</v>
       </c>
@@ -5865,7 +5865,7 @@
       <c r="AE19" s="2"/>
       <c r="AF19" s="40"/>
     </row>
-    <row r="20" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B20" s="11">
         <v>2</v>
       </c>
@@ -5920,7 +5920,7 @@
       <c r="AE20" s="2"/>
       <c r="AF20" s="40"/>
     </row>
-    <row r="21" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B21" s="11">
         <v>2</v>
       </c>
@@ -5975,7 +5975,7 @@
       <c r="AE21" s="2"/>
       <c r="AF21" s="40"/>
     </row>
-    <row r="22" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B22" s="11">
         <v>2</v>
       </c>
@@ -6030,7 +6030,7 @@
       <c r="AE22" s="2"/>
       <c r="AF22" s="40"/>
     </row>
-    <row r="23" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B23" s="13">
         <v>2</v>
       </c>
@@ -6097,7 +6097,7 @@
       <c r="AE23" s="2"/>
       <c r="AF23" s="40"/>
     </row>
-    <row r="24" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B24" s="6">
         <v>3</v>
       </c>
@@ -6185,7 +6185,7 @@
         <v>16.341485802915539</v>
       </c>
     </row>
-    <row r="25" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B25" s="11">
         <v>3</v>
       </c>
@@ -6242,7 +6242,7 @@
       <c r="AE25" s="28"/>
       <c r="AF25" s="39"/>
     </row>
-    <row r="26" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B26" s="11">
         <v>3</v>
       </c>
@@ -6299,7 +6299,7 @@
       <c r="AE26" s="2"/>
       <c r="AF26" s="40"/>
     </row>
-    <row r="27" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B27" s="11">
         <v>3</v>
       </c>
@@ -6356,7 +6356,7 @@
       <c r="AE27" s="2"/>
       <c r="AF27" s="40"/>
     </row>
-    <row r="28" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B28" s="11">
         <v>3</v>
       </c>
@@ -6413,7 +6413,7 @@
       <c r="AE28" s="2"/>
       <c r="AF28" s="40"/>
     </row>
-    <row r="29" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B29" s="11">
         <v>3</v>
       </c>
@@ -6470,7 +6470,7 @@
       <c r="AE29" s="2"/>
       <c r="AF29" s="40"/>
     </row>
-    <row r="30" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B30" s="11">
         <v>3</v>
       </c>
@@ -6527,7 +6527,7 @@
       <c r="AE30" s="2"/>
       <c r="AF30" s="40"/>
     </row>
-    <row r="31" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B31" s="11">
         <v>3</v>
       </c>
@@ -6584,7 +6584,7 @@
       <c r="AE31" s="2"/>
       <c r="AF31" s="40"/>
     </row>
-    <row r="32" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B32" s="11">
         <v>3</v>
       </c>
@@ -6650,7 +6650,7 @@
         <v>11.995541941166838</v>
       </c>
     </row>
-    <row r="33" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B33" s="13">
         <v>3</v>
       </c>
@@ -6719,7 +6719,7 @@
       <c r="AE33" s="28"/>
       <c r="AF33" s="39"/>
     </row>
-    <row r="34" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B34" s="11">
         <v>4</v>
       </c>
@@ -6798,7 +6798,7 @@
       <c r="AE34" s="2"/>
       <c r="AF34" s="40"/>
     </row>
-    <row r="35" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B35" s="11">
         <v>4</v>
       </c>
@@ -6853,7 +6853,7 @@
       <c r="AE35" s="2"/>
       <c r="AF35" s="40"/>
     </row>
-    <row r="36" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B36" s="11">
         <v>4</v>
       </c>
@@ -6917,7 +6917,7 @@
         <v>13.592134752219362</v>
       </c>
     </row>
-    <row r="37" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B37" s="11">
         <v>4</v>
       </c>
@@ -6974,7 +6974,7 @@
         <v>14.430505770348006</v>
       </c>
     </row>
-    <row r="38" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B38" s="11">
         <v>4</v>
       </c>
@@ -7034,7 +7034,7 @@
         <v>11.780184646827356</v>
       </c>
     </row>
-    <row r="39" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B39" s="13">
         <v>4</v>
       </c>
@@ -7106,7 +7106,7 @@
         <v>18.399887376710556</v>
       </c>
     </row>
-    <row r="40" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B40" s="43" t="s">
         <v>11</v>
       </c>
@@ -7174,7 +7174,7 @@
         <v>11.248660267146384</v>
       </c>
     </row>
-    <row r="41" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B41" t="s">
         <v>12</v>
       </c>
@@ -7221,7 +7221,7 @@
         <v>10.704819498388627</v>
       </c>
     </row>
-    <row r="42" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B42" s="44" t="s">
         <v>13</v>
       </c>
@@ -7274,7 +7274,7 @@
       </c>
       <c r="AB42" s="3"/>
     </row>
-    <row r="43" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:32" x14ac:dyDescent="0.35">
       <c r="J43" s="44" t="s">
         <v>13</v>
       </c>
@@ -7312,7 +7312,7 @@
         <v>12.890736472214234</v>
       </c>
     </row>
-    <row r="47" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B47" s="22"/>
       <c r="C47" s="17"/>
       <c r="D47" s="17"/>
@@ -7341,7 +7341,7 @@
       <c r="W47" s="17"/>
       <c r="X47" s="18"/>
     </row>
-    <row r="48" spans="2:32" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:32" x14ac:dyDescent="0.35">
       <c r="B48" s="13" t="s">
         <v>1</v>
       </c>
@@ -7406,7 +7406,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="49" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B49" s="6">
         <v>1</v>
       </c>
@@ -7447,7 +7447,7 @@
       <c r="W49" s="28"/>
       <c r="X49" s="39"/>
     </row>
-    <row r="50" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B50" s="11">
         <v>1</v>
       </c>
@@ -7488,7 +7488,7 @@
       <c r="W50" s="2"/>
       <c r="X50" s="40"/>
     </row>
-    <row r="51" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B51" s="11">
         <v>1</v>
       </c>
@@ -7529,7 +7529,7 @@
       <c r="W51" s="2"/>
       <c r="X51" s="40"/>
     </row>
-    <row r="52" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B52" s="11">
         <v>1</v>
       </c>
@@ -7570,7 +7570,7 @@
       <c r="W52" s="2"/>
       <c r="X52" s="40"/>
     </row>
-    <row r="53" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B53" s="11">
         <v>1</v>
       </c>
@@ -7611,7 +7611,7 @@
       <c r="W53" s="2"/>
       <c r="X53" s="40"/>
     </row>
-    <row r="54" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B54" s="11">
         <v>1</v>
       </c>
@@ -7652,7 +7652,7 @@
       <c r="W54" s="2"/>
       <c r="X54" s="40"/>
     </row>
-    <row r="55" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B55" s="11">
         <v>1</v>
       </c>
@@ -7693,7 +7693,7 @@
       <c r="W55" s="2"/>
       <c r="X55" s="40"/>
     </row>
-    <row r="56" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B56" s="11">
         <v>1</v>
       </c>
@@ -7734,7 +7734,7 @@
       <c r="W56" s="2"/>
       <c r="X56" s="40"/>
     </row>
-    <row r="57" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B57" s="11">
         <v>1</v>
       </c>
@@ -7775,7 +7775,7 @@
       <c r="W57" s="2"/>
       <c r="X57" s="40"/>
     </row>
-    <row r="58" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B58" s="13">
         <v>1</v>
       </c>
@@ -7852,7 +7852,7 @@
         <v>12.467552636726225</v>
       </c>
     </row>
-    <row r="59" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B59" s="6">
         <v>2</v>
       </c>
@@ -7893,7 +7893,7 @@
       <c r="W59" s="28"/>
       <c r="X59" s="39"/>
     </row>
-    <row r="60" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B60" s="11">
         <v>2</v>
       </c>
@@ -7934,7 +7934,7 @@
       <c r="W60" s="2"/>
       <c r="X60" s="40"/>
     </row>
-    <row r="61" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B61" s="11">
         <v>2</v>
       </c>
@@ -7975,7 +7975,7 @@
       <c r="W61" s="2"/>
       <c r="X61" s="40"/>
     </row>
-    <row r="62" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B62" s="11">
         <v>2</v>
       </c>
@@ -8016,7 +8016,7 @@
       <c r="W62" s="2"/>
       <c r="X62" s="40"/>
     </row>
-    <row r="63" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B63" s="11">
         <v>2</v>
       </c>
@@ -8057,7 +8057,7 @@
       <c r="W63" s="2"/>
       <c r="X63" s="40"/>
     </row>
-    <row r="64" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B64" s="11">
         <v>2</v>
       </c>
@@ -8098,7 +8098,7 @@
       <c r="W64" s="2"/>
       <c r="X64" s="40"/>
     </row>
-    <row r="65" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B65" s="11">
         <v>2</v>
       </c>
@@ -8139,7 +8139,7 @@
       <c r="W65" s="2"/>
       <c r="X65" s="40"/>
     </row>
-    <row r="66" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B66" s="11">
         <v>2</v>
       </c>
@@ -8180,7 +8180,7 @@
       <c r="W66" s="2"/>
       <c r="X66" s="40"/>
     </row>
-    <row r="67" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B67" s="11">
         <v>2</v>
       </c>
@@ -8221,7 +8221,7 @@
       <c r="W67" s="2"/>
       <c r="X67" s="40"/>
     </row>
-    <row r="68" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B68" s="13">
         <v>2</v>
       </c>
@@ -8298,7 +8298,7 @@
         <v>14.19505253988679</v>
       </c>
     </row>
-    <row r="69" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B69" s="6">
         <v>3</v>
       </c>
@@ -8339,7 +8339,7 @@
       <c r="W69" s="28"/>
       <c r="X69" s="39"/>
     </row>
-    <row r="70" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B70" s="11">
         <v>3</v>
       </c>
@@ -8380,7 +8380,7 @@
       <c r="W70" s="2"/>
       <c r="X70" s="40"/>
     </row>
-    <row r="71" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B71" s="11">
         <v>3</v>
       </c>
@@ -8421,7 +8421,7 @@
       <c r="W71" s="2"/>
       <c r="X71" s="40"/>
     </row>
-    <row r="72" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B72" s="11">
         <v>3</v>
       </c>
@@ -8462,7 +8462,7 @@
       <c r="W72" s="2"/>
       <c r="X72" s="40"/>
     </row>
-    <row r="73" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B73" s="11">
         <v>3</v>
       </c>
@@ -8503,7 +8503,7 @@
       <c r="W73" s="2"/>
       <c r="X73" s="40"/>
     </row>
-    <row r="74" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B74" s="11">
         <v>3</v>
       </c>
@@ -8544,7 +8544,7 @@
       <c r="W74" s="2"/>
       <c r="X74" s="40"/>
     </row>
-    <row r="75" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B75" s="11">
         <v>3</v>
       </c>
@@ -8585,7 +8585,7 @@
       <c r="W75" s="2"/>
       <c r="X75" s="40"/>
     </row>
-    <row r="76" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B76" s="11">
         <v>3</v>
       </c>
@@ -8626,7 +8626,7 @@
       <c r="W76" s="2"/>
       <c r="X76" s="40"/>
     </row>
-    <row r="77" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B77" s="11">
         <v>3</v>
       </c>
@@ -8667,7 +8667,7 @@
       <c r="W77" s="2"/>
       <c r="X77" s="40"/>
     </row>
-    <row r="78" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B78" s="13">
         <v>3</v>
       </c>
@@ -8744,7 +8744,7 @@
         <v>13.739374608186964</v>
       </c>
     </row>
-    <row r="79" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B79" s="43" t="s">
         <v>11</v>
       </c>
@@ -8791,7 +8791,7 @@
         <v>13.467326594933326</v>
       </c>
     </row>
-    <row r="80" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B80" t="s">
         <v>12</v>
       </c>
@@ -8850,7 +8850,7 @@
         <v>3.7875326427181033</v>
       </c>
     </row>
-    <row r="81" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B81" s="44" t="s">
         <v>13</v>
       </c>
@@ -8924,22 +8924,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48E976A1-F91A-48C1-BCAD-1333CCE54E38}">
   <dimension ref="A1:M346"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="29.28515625" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" customWidth="1"/>
-    <col min="3" max="3" width="27.5703125" customWidth="1"/>
-    <col min="5" max="5" width="8.85546875" customWidth="1"/>
-    <col min="7" max="7" width="9.85546875" customWidth="1"/>
-    <col min="8" max="8" width="13.42578125" customWidth="1"/>
+    <col min="1" max="1" width="29.26953125" customWidth="1"/>
+    <col min="2" max="2" width="10.1796875" customWidth="1"/>
+    <col min="3" max="3" width="27.54296875" customWidth="1"/>
+    <col min="5" max="5" width="8.81640625" customWidth="1"/>
+    <col min="7" max="7" width="9.81640625" customWidth="1"/>
+    <col min="8" max="8" width="13.453125" customWidth="1"/>
     <col min="9" max="9" width="15" customWidth="1"/>
-    <col min="10" max="10" width="31.85546875" customWidth="1"/>
-    <col min="11" max="11" width="35.85546875" customWidth="1"/>
-    <col min="12" max="12" width="26.140625" customWidth="1"/>
-    <col min="13" max="13" width="10.140625" customWidth="1"/>
+    <col min="10" max="10" width="31.81640625" customWidth="1"/>
+    <col min="11" max="11" width="35.81640625" customWidth="1"/>
+    <col min="12" max="12" width="26.1796875" customWidth="1"/>
+    <col min="13" max="13" width="10.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>42</v>
       </c>
@@ -8980,7 +8980,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>35</v>
       </c>
@@ -9015,7 +9015,7 @@
         <v>85.753100000000003</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>35</v>
       </c>
@@ -9050,7 +9050,7 @@
         <v>17.744</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -9085,7 +9085,7 @@
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>35</v>
       </c>
@@ -9120,7 +9120,7 @@
         <v>2.4927000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>35</v>
       </c>
@@ -9155,7 +9155,7 @@
         <v>2060.8047999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>35</v>
       </c>
@@ -9190,7 +9190,7 @@
         <v>2060.8047999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>35</v>
       </c>
@@ -9225,7 +9225,7 @@
         <v>1.6526000000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>35</v>
       </c>
@@ -9260,7 +9260,7 @@
         <v>85.753100000000003</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>35</v>
       </c>
@@ -9295,7 +9295,7 @@
         <v>17.744</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>35</v>
       </c>
@@ -9330,7 +9330,7 @@
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>35</v>
       </c>
@@ -9365,7 +9365,7 @@
         <v>2.4927000000000001</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>35</v>
       </c>
@@ -9400,7 +9400,7 @@
         <v>1.6526000000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>35</v>
       </c>
@@ -9435,7 +9435,7 @@
         <v>85.753100000000003</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>35</v>
       </c>
@@ -9470,7 +9470,7 @@
         <v>17.744</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>35</v>
       </c>
@@ -9505,7 +9505,7 @@
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>35</v>
       </c>
@@ -9540,7 +9540,7 @@
         <v>2.4927000000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>35</v>
       </c>
@@ -9575,7 +9575,7 @@
         <v>408.40640000000002</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>35</v>
       </c>
@@ -9610,7 +9610,7 @@
         <v>408.40640000000002</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>35</v>
       </c>
@@ -9645,7 +9645,7 @@
         <v>1.6526000000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>35</v>
       </c>
@@ -9680,7 +9680,7 @@
         <v>85.753100000000003</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>35</v>
       </c>
@@ -9715,7 +9715,7 @@
         <v>17.744</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>35</v>
       </c>
@@ -9750,7 +9750,7 @@
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>35</v>
       </c>
@@ -9785,7 +9785,7 @@
         <v>2.4927000000000001</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>35</v>
       </c>
@@ -9820,7 +9820,7 @@
         <v>1.6526000000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>35</v>
       </c>
@@ -9855,7 +9855,7 @@
         <v>85.753100000000003</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>35</v>
       </c>
@@ -9890,7 +9890,7 @@
         <v>5.7873000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>35</v>
       </c>
@@ -9925,7 +9925,7 @@
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>35</v>
       </c>
@@ -9960,7 +9960,7 @@
         <v>65.186000000000007</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>35</v>
       </c>
@@ -9995,7 +9995,7 @@
         <v>81.382000000000005</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>35</v>
       </c>
@@ -10030,7 +10030,7 @@
         <v>81.382000000000005</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>35</v>
       </c>
@@ -10065,7 +10065,7 @@
         <v>1.6526000000000001</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>35</v>
       </c>
@@ -10100,7 +10100,7 @@
         <v>85.753100000000003</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>35</v>
       </c>
@@ -10135,7 +10135,7 @@
         <v>5.7873000000000001</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>35</v>
       </c>
@@ -10170,7 +10170,7 @@
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>35</v>
       </c>
@@ -10205,7 +10205,7 @@
         <v>65.186000000000007</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>35</v>
       </c>
@@ -10240,7 +10240,7 @@
         <v>1.6526000000000001</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>35</v>
       </c>
@@ -10275,7 +10275,7 @@
         <v>85.753100000000003</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>35</v>
       </c>
@@ -10310,7 +10310,7 @@
         <v>5.7873000000000001</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>35</v>
       </c>
@@ -10345,7 +10345,7 @@
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>35</v>
       </c>
@@ -10380,7 +10380,7 @@
         <v>65.186000000000007</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>35</v>
       </c>
@@ -10415,7 +10415,7 @@
         <v>14.942</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>35</v>
       </c>
@@ -10450,7 +10450,7 @@
         <v>14.942</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>35</v>
       </c>
@@ -10485,7 +10485,7 @@
         <v>1.6526000000000001</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>35</v>
       </c>
@@ -10520,7 +10520,7 @@
         <v>85.753100000000003</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>35</v>
       </c>
@@ -10555,7 +10555,7 @@
         <v>5.7873000000000001</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>35</v>
       </c>
@@ -10590,7 +10590,7 @@
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>35</v>
       </c>
@@ -10625,7 +10625,7 @@
         <v>65.186000000000007</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>35</v>
       </c>
@@ -10660,7 +10660,7 @@
         <v>1.6526000000000001</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>35</v>
       </c>
@@ -10695,7 +10695,7 @@
         <v>85.753100000000003</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>35</v>
       </c>
@@ -10730,7 +10730,7 @@
         <v>5.7873000000000001</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>35</v>
       </c>
@@ -10765,7 +10765,7 @@
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>35</v>
       </c>
@@ -10800,7 +10800,7 @@
         <v>65.186000000000007</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>35</v>
       </c>
@@ -10835,7 +10835,7 @@
         <v>3.0041000000000002</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>35</v>
       </c>
@@ -10870,7 +10870,7 @@
         <v>3.0041000000000002</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>35</v>
       </c>
@@ -10905,7 +10905,7 @@
         <v>1.6526000000000001</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>35</v>
       </c>
@@ -10940,7 +10940,7 @@
         <v>85.753100000000003</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>35</v>
       </c>
@@ -10975,7 +10975,7 @@
         <v>5.7873000000000001</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>35</v>
       </c>
@@ -11010,7 +11010,7 @@
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>35</v>
       </c>
@@ -11045,7 +11045,7 @@
         <v>65.186000000000007</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>35</v>
       </c>
@@ -11080,7 +11080,7 @@
         <v>1.6526000000000001</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>35</v>
       </c>
@@ -11115,7 +11115,7 @@
         <v>17.744</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>35</v>
       </c>
@@ -11150,7 +11150,7 @@
         <v>5.7873000000000001</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>35</v>
       </c>
@@ -11185,7 +11185,7 @@
         <v>2.4927000000000001</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>35</v>
       </c>
@@ -11220,7 +11220,7 @@
         <v>65.186000000000007</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>35</v>
       </c>
@@ -11255,7 +11255,7 @@
         <v>0.62690000000000001</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>35</v>
       </c>
@@ -11290,7 +11290,7 @@
         <v>0.62690000000000001</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>35</v>
       </c>
@@ -11325,7 +11325,7 @@
         <v>8.6E-3</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>35</v>
       </c>
@@ -11360,7 +11360,7 @@
         <v>17.744</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>35</v>
       </c>
@@ -11395,7 +11395,7 @@
         <v>5.7873000000000001</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>35</v>
       </c>
@@ -11430,7 +11430,7 @@
         <v>2.4927000000000001</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>35</v>
       </c>
@@ -11465,7 +11465,7 @@
         <v>65.186000000000007</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>35</v>
       </c>
@@ -11500,7 +11500,7 @@
         <v>8.6E-3</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>35</v>
       </c>
@@ -11535,7 +11535,7 @@
         <v>17.744</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>35</v>
       </c>
@@ -11570,7 +11570,7 @@
         <v>5.7873000000000001</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>35</v>
       </c>
@@ -11605,7 +11605,7 @@
         <v>2.4927000000000001</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>35</v>
       </c>
@@ -11640,7 +11640,7 @@
         <v>65.186000000000007</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>35</v>
       </c>
@@ -11675,7 +11675,7 @@
         <v>0.13930000000000001</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>35</v>
       </c>
@@ -11710,7 +11710,7 @@
         <v>0.13930000000000001</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>35</v>
       </c>
@@ -11745,7 +11745,7 @@
         <v>8.6E-3</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>35</v>
       </c>
@@ -11780,7 +11780,7 @@
         <v>17.744</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>35</v>
       </c>
@@ -11815,7 +11815,7 @@
         <v>5.7873000000000001</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>35</v>
       </c>
@@ -11850,7 +11850,7 @@
         <v>2.4927000000000001</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>35</v>
       </c>
@@ -11885,7 +11885,7 @@
         <v>65.186000000000007</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>35</v>
       </c>
@@ -11920,7 +11920,7 @@
         <v>8.6E-3</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>35</v>
       </c>
@@ -11955,7 +11955,7 @@
         <v>17.744</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>35</v>
       </c>
@@ -11990,7 +11990,7 @@
         <v>8.6E-3</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>35</v>
       </c>
@@ -12025,7 +12025,7 @@
         <v>2.4927000000000001</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>35</v>
       </c>
@@ -12060,7 +12060,7 @@
         <v>8.6E-3</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>35</v>
       </c>
@@ -12095,7 +12095,7 @@
         <v>8.0999999999999996E-3</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>35</v>
       </c>
@@ -12130,7 +12130,7 @@
         <v>8.0999999999999996E-3</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>35</v>
       </c>
@@ -12165,7 +12165,7 @@
         <v>8.6E-3</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>35</v>
       </c>
@@ -12200,7 +12200,7 @@
         <v>17.744</v>
       </c>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>35</v>
       </c>
@@ -12235,7 +12235,7 @@
         <v>8.6E-3</v>
       </c>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>35</v>
       </c>
@@ -12270,7 +12270,7 @@
         <v>2.4927000000000001</v>
       </c>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>35</v>
       </c>
@@ -12305,7 +12305,7 @@
         <v>8.6E-3</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>35</v>
       </c>
@@ -12340,7 +12340,7 @@
         <v>8.6E-3</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>34</v>
       </c>
@@ -12375,7 +12375,7 @@
         <v>100.6874</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>34</v>
       </c>
@@ -12410,7 +12410,7 @@
         <v>20.672799999999999</v>
       </c>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>34</v>
       </c>
@@ -12445,7 +12445,7 @@
         <v>9.06E-2</v>
       </c>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>34</v>
       </c>
@@ -12480,7 +12480,7 @@
         <v>2.8092999999999999</v>
       </c>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>34</v>
       </c>
@@ -12515,7 +12515,7 @@
         <v>1947.9368999999999</v>
       </c>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>34</v>
       </c>
@@ -12550,7 +12550,7 @@
         <v>1947.9368999999999</v>
       </c>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>34</v>
       </c>
@@ -12585,7 +12585,7 @@
         <v>2.1316999999999999</v>
       </c>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>34</v>
       </c>
@@ -12620,7 +12620,7 @@
         <v>100.6874</v>
       </c>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>34</v>
       </c>
@@ -12655,7 +12655,7 @@
         <v>20.672799999999999</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>34</v>
       </c>
@@ -12690,7 +12690,7 @@
         <v>9.06E-2</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>34</v>
       </c>
@@ -12725,7 +12725,7 @@
         <v>2.8092999999999999</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>34</v>
       </c>
@@ -12760,7 +12760,7 @@
         <v>2.1316999999999999</v>
       </c>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>34</v>
       </c>
@@ -12795,7 +12795,7 @@
         <v>100.6874</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>34</v>
       </c>
@@ -12830,7 +12830,7 @@
         <v>20.672799999999999</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>34</v>
       </c>
@@ -12865,7 +12865,7 @@
         <v>9.06E-2</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>34</v>
       </c>
@@ -12900,7 +12900,7 @@
         <v>2.8092999999999999</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>34</v>
       </c>
@@ -12935,7 +12935,7 @@
         <v>408.173</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>34</v>
       </c>
@@ -12970,7 +12970,7 @@
         <v>408.173</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>34</v>
       </c>
@@ -13005,7 +13005,7 @@
         <v>2.1316999999999999</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>34</v>
       </c>
@@ -13040,7 +13040,7 @@
         <v>100.6874</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>34</v>
       </c>
@@ -13075,7 +13075,7 @@
         <v>20.672799999999999</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>34</v>
       </c>
@@ -13110,7 +13110,7 @@
         <v>9.06E-2</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>34</v>
       </c>
@@ -13145,7 +13145,7 @@
         <v>2.8092999999999999</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>34</v>
       </c>
@@ -13180,7 +13180,7 @@
         <v>2.1316999999999999</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>34</v>
       </c>
@@ -13215,7 +13215,7 @@
         <v>6.8619000000000003</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>34</v>
       </c>
@@ -13250,7 +13250,7 @@
         <v>9.06E-2</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>34</v>
       </c>
@@ -13285,7 +13285,7 @@
         <v>71.095200000000006</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>34</v>
       </c>
@@ -13320,7 +13320,7 @@
         <v>82.256699999999995</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>34</v>
       </c>
@@ -13355,7 +13355,7 @@
         <v>82.256699999999995</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>34</v>
       </c>
@@ -13390,7 +13390,7 @@
         <v>2.1316999999999999</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>34</v>
       </c>
@@ -13425,7 +13425,7 @@
         <v>100.6874</v>
       </c>
     </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>34</v>
       </c>
@@ -13460,7 +13460,7 @@
         <v>6.8619000000000003</v>
       </c>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>34</v>
       </c>
@@ -13495,7 +13495,7 @@
         <v>9.06E-2</v>
       </c>
     </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>34</v>
       </c>
@@ -13530,7 +13530,7 @@
         <v>71.095200000000006</v>
       </c>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>34</v>
       </c>
@@ -13565,7 +13565,7 @@
         <v>2.1316999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>34</v>
       </c>
@@ -13600,7 +13600,7 @@
         <v>100.6874</v>
       </c>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>34</v>
       </c>
@@ -13635,7 +13635,7 @@
         <v>6.8619000000000003</v>
       </c>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>34</v>
       </c>
@@ -13670,7 +13670,7 @@
         <v>9.06E-2</v>
       </c>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>34</v>
       </c>
@@ -13705,7 +13705,7 @@
         <v>71.095200000000006</v>
       </c>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>34</v>
       </c>
@@ -13740,7 +13740,7 @@
         <v>16.223700000000001</v>
       </c>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>34</v>
       </c>
@@ -13775,7 +13775,7 @@
         <v>16.223700000000001</v>
       </c>
     </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>34</v>
       </c>
@@ -13810,7 +13810,7 @@
         <v>2.1316999999999999</v>
       </c>
     </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>34</v>
       </c>
@@ -13845,7 +13845,7 @@
         <v>100.6874</v>
       </c>
     </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>34</v>
       </c>
@@ -13880,7 +13880,7 @@
         <v>6.8619000000000003</v>
       </c>
     </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>34</v>
       </c>
@@ -13915,7 +13915,7 @@
         <v>9.06E-2</v>
       </c>
     </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>34</v>
       </c>
@@ -13950,7 +13950,7 @@
         <v>71.095200000000006</v>
       </c>
     </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>34</v>
       </c>
@@ -13985,7 +13985,7 @@
         <v>2.1316999999999999</v>
       </c>
     </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>34</v>
       </c>
@@ -14020,7 +14020,7 @@
         <v>100.6874</v>
       </c>
     </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>34</v>
       </c>
@@ -14055,7 +14055,7 @@
         <v>6.8619000000000003</v>
       </c>
     </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>34</v>
       </c>
@@ -14090,7 +14090,7 @@
         <v>9.06E-2</v>
       </c>
     </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>34</v>
       </c>
@@ -14125,7 +14125,7 @@
         <v>71.095200000000006</v>
       </c>
     </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>34</v>
       </c>
@@ -14160,7 +14160,7 @@
         <v>3.3439999999999999</v>
       </c>
     </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>34</v>
       </c>
@@ -14195,7 +14195,7 @@
         <v>3.3439999999999999</v>
       </c>
     </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>34</v>
       </c>
@@ -14230,7 +14230,7 @@
         <v>2.1316999999999999</v>
       </c>
     </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>34</v>
       </c>
@@ -14265,7 +14265,7 @@
         <v>100.6874</v>
       </c>
     </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>34</v>
       </c>
@@ -14300,7 +14300,7 @@
         <v>6.8619000000000003</v>
       </c>
     </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>34</v>
       </c>
@@ -14335,7 +14335,7 @@
         <v>9.06E-2</v>
       </c>
     </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>34</v>
       </c>
@@ -14370,7 +14370,7 @@
         <v>71.095200000000006</v>
       </c>
     </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>34</v>
       </c>
@@ -14405,7 +14405,7 @@
         <v>2.1316999999999999</v>
       </c>
     </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>34</v>
       </c>
@@ -14440,7 +14440,7 @@
         <v>20.672799999999999</v>
       </c>
     </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>34</v>
       </c>
@@ -14475,7 +14475,7 @@
         <v>6.8619000000000003</v>
       </c>
     </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>34</v>
       </c>
@@ -14510,7 +14510,7 @@
         <v>2.8092999999999999</v>
       </c>
     </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>34</v>
       </c>
@@ -14545,7 +14545,7 @@
         <v>71.095200000000006</v>
       </c>
     </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>34</v>
       </c>
@@ -14580,7 +14580,7 @@
         <v>0.53249999999999997</v>
       </c>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>34</v>
       </c>
@@ -14615,7 +14615,7 @@
         <v>0.53249999999999997</v>
       </c>
     </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>34</v>
       </c>
@@ -14650,7 +14650,7 @@
         <v>6.8999999999999999E-3</v>
       </c>
     </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>34</v>
       </c>
@@ -14685,7 +14685,7 @@
         <v>20.672799999999999</v>
       </c>
     </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>34</v>
       </c>
@@ -14720,7 +14720,7 @@
         <v>6.8619000000000003</v>
       </c>
     </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>34</v>
       </c>
@@ -14755,7 +14755,7 @@
         <v>2.8092999999999999</v>
       </c>
     </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>34</v>
       </c>
@@ -14790,7 +14790,7 @@
         <v>71.095200000000006</v>
       </c>
     </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>34</v>
       </c>
@@ -14825,7 +14825,7 @@
         <v>6.8999999999999999E-3</v>
       </c>
     </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>34</v>
       </c>
@@ -14860,7 +14860,7 @@
         <v>20.672799999999999</v>
       </c>
     </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>34</v>
       </c>
@@ -14895,7 +14895,7 @@
         <v>6.8619000000000003</v>
       </c>
     </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>34</v>
       </c>
@@ -14930,7 +14930,7 @@
         <v>2.8092999999999999</v>
       </c>
     </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>34</v>
       </c>
@@ -14965,7 +14965,7 @@
         <v>71.095200000000006</v>
       </c>
     </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>34</v>
       </c>
@@ -15000,7 +15000,7 @@
         <v>0.1421</v>
       </c>
     </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>34</v>
       </c>
@@ -15035,7 +15035,7 @@
         <v>0.1421</v>
       </c>
     </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>34</v>
       </c>
@@ -15070,7 +15070,7 @@
         <v>6.8999999999999999E-3</v>
       </c>
     </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>34</v>
       </c>
@@ -15105,7 +15105,7 @@
         <v>20.672799999999999</v>
       </c>
     </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>34</v>
       </c>
@@ -15140,7 +15140,7 @@
         <v>6.8619000000000003</v>
       </c>
     </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>34</v>
       </c>
@@ -15175,7 +15175,7 @@
         <v>2.8092999999999999</v>
       </c>
     </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>34</v>
       </c>
@@ -15210,7 +15210,7 @@
         <v>71.095200000000006</v>
       </c>
     </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
         <v>34</v>
       </c>
@@ -15245,7 +15245,7 @@
         <v>6.8999999999999999E-3</v>
       </c>
     </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
         <v>34</v>
       </c>
@@ -15280,7 +15280,7 @@
         <v>20.672799999999999</v>
       </c>
     </row>
-    <row r="182" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>34</v>
       </c>
@@ -15315,7 +15315,7 @@
         <v>6.8999999999999999E-3</v>
       </c>
     </row>
-    <row r="183" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>34</v>
       </c>
@@ -15350,7 +15350,7 @@
         <v>2.8092999999999999</v>
       </c>
     </row>
-    <row r="184" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>34</v>
       </c>
@@ -15385,7 +15385,7 @@
         <v>6.8999999999999999E-3</v>
       </c>
     </row>
-    <row r="185" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
         <v>34</v>
       </c>
@@ -15420,7 +15420,7 @@
         <v>8.3999999999999995E-3</v>
       </c>
     </row>
-    <row r="186" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
         <v>34</v>
       </c>
@@ -15455,7 +15455,7 @@
         <v>8.3999999999999995E-3</v>
       </c>
     </row>
-    <row r="187" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
         <v>34</v>
       </c>
@@ -15490,7 +15490,7 @@
         <v>6.8999999999999999E-3</v>
       </c>
     </row>
-    <row r="188" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
         <v>34</v>
       </c>
@@ -15525,7 +15525,7 @@
         <v>20.672799999999999</v>
       </c>
     </row>
-    <row r="189" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
         <v>34</v>
       </c>
@@ -15560,7 +15560,7 @@
         <v>6.8999999999999999E-3</v>
       </c>
     </row>
-    <row r="190" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
         <v>34</v>
       </c>
@@ -15595,7 +15595,7 @@
         <v>2.8092999999999999</v>
       </c>
     </row>
-    <row r="191" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
         <v>34</v>
       </c>
@@ -15630,7 +15630,7 @@
         <v>6.8999999999999999E-3</v>
       </c>
     </row>
-    <row r="192" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>34</v>
       </c>
@@ -15665,7 +15665,7 @@
         <v>6.8999999999999999E-3</v>
       </c>
     </row>
-    <row r="193" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>33</v>
       </c>
@@ -15700,7 +15700,7 @@
         <v>85.823300000000003</v>
       </c>
     </row>
-    <row r="194" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>33</v>
       </c>
@@ -15735,7 +15735,7 @@
         <v>18.533899999999999</v>
       </c>
     </row>
-    <row r="195" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>33</v>
       </c>
@@ -15770,7 +15770,7 @@
         <v>8.5000000000000006E-2</v>
       </c>
     </row>
-    <row r="196" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
         <v>33</v>
       </c>
@@ -15805,7 +15805,7 @@
         <v>2.4902000000000002</v>
       </c>
     </row>
-    <row r="197" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>33</v>
       </c>
@@ -15840,7 +15840,7 @@
         <v>1944.2019</v>
       </c>
     </row>
-    <row r="198" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
         <v>33</v>
       </c>
@@ -15875,7 +15875,7 @@
         <v>1944.2019</v>
       </c>
     </row>
-    <row r="199" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
         <v>33</v>
       </c>
@@ -15910,7 +15910,7 @@
         <v>1.7131000000000001</v>
       </c>
     </row>
-    <row r="200" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>33</v>
       </c>
@@ -15945,7 +15945,7 @@
         <v>85.823300000000003</v>
       </c>
     </row>
-    <row r="201" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
         <v>33</v>
       </c>
@@ -15980,7 +15980,7 @@
         <v>18.533899999999999</v>
       </c>
     </row>
-    <row r="202" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
         <v>33</v>
       </c>
@@ -16015,7 +16015,7 @@
         <v>8.5000000000000006E-2</v>
       </c>
     </row>
-    <row r="203" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
         <v>33</v>
       </c>
@@ -16050,7 +16050,7 @@
         <v>2.4902000000000002</v>
       </c>
     </row>
-    <row r="204" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
         <v>33</v>
       </c>
@@ -16085,7 +16085,7 @@
         <v>1.7131000000000001</v>
       </c>
     </row>
-    <row r="205" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
         <v>33</v>
       </c>
@@ -16120,7 +16120,7 @@
         <v>85.823300000000003</v>
       </c>
     </row>
-    <row r="206" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
         <v>33</v>
       </c>
@@ -16155,7 +16155,7 @@
         <v>18.533899999999999</v>
       </c>
     </row>
-    <row r="207" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
         <v>33</v>
       </c>
@@ -16190,7 +16190,7 @@
         <v>8.5000000000000006E-2</v>
       </c>
     </row>
-    <row r="208" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
         <v>33</v>
       </c>
@@ -16225,7 +16225,7 @@
         <v>2.4902000000000002</v>
       </c>
     </row>
-    <row r="209" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
         <v>33</v>
       </c>
@@ -16260,7 +16260,7 @@
         <v>401.23020000000002</v>
       </c>
     </row>
-    <row r="210" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
         <v>33</v>
       </c>
@@ -16295,7 +16295,7 @@
         <v>401.23020000000002</v>
       </c>
     </row>
-    <row r="211" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
         <v>33</v>
       </c>
@@ -16330,7 +16330,7 @@
         <v>1.7131000000000001</v>
       </c>
     </row>
-    <row r="212" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
         <v>33</v>
       </c>
@@ -16365,7 +16365,7 @@
         <v>85.823300000000003</v>
       </c>
     </row>
-    <row r="213" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
         <v>33</v>
       </c>
@@ -16400,7 +16400,7 @@
         <v>18.533899999999999</v>
       </c>
     </row>
-    <row r="214" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
         <v>33</v>
       </c>
@@ -16435,7 +16435,7 @@
         <v>8.5000000000000006E-2</v>
       </c>
     </row>
-    <row r="215" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
         <v>33</v>
       </c>
@@ -16470,7 +16470,7 @@
         <v>2.4902000000000002</v>
       </c>
     </row>
-    <row r="216" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
         <v>33</v>
       </c>
@@ -16505,7 +16505,7 @@
         <v>1.7131000000000001</v>
       </c>
     </row>
-    <row r="217" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
         <v>33</v>
       </c>
@@ -16540,7 +16540,7 @@
         <v>85.823300000000003</v>
       </c>
     </row>
-    <row r="218" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
         <v>33</v>
       </c>
@@ -16575,7 +16575,7 @@
         <v>5.9260999999999999</v>
       </c>
     </row>
-    <row r="219" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
         <v>33</v>
       </c>
@@ -16610,7 +16610,7 @@
         <v>8.5000000000000006E-2</v>
       </c>
     </row>
-    <row r="220" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
         <v>33</v>
       </c>
@@ -16645,7 +16645,7 @@
         <v>65.522800000000004</v>
       </c>
     </row>
-    <row r="221" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
         <v>33</v>
       </c>
@@ -16680,7 +16680,7 @@
         <v>81.263599999999997</v>
       </c>
     </row>
-    <row r="222" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
         <v>33</v>
       </c>
@@ -16715,7 +16715,7 @@
         <v>81.263599999999997</v>
       </c>
     </row>
-    <row r="223" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
         <v>33</v>
       </c>
@@ -16750,7 +16750,7 @@
         <v>85.823300000000003</v>
       </c>
     </row>
-    <row r="224" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
         <v>33</v>
       </c>
@@ -16785,7 +16785,7 @@
         <v>5.9260999999999999</v>
       </c>
     </row>
-    <row r="225" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>33</v>
       </c>
@@ -16820,7 +16820,7 @@
         <v>8.5000000000000006E-2</v>
       </c>
     </row>
-    <row r="226" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
         <v>33</v>
       </c>
@@ -16855,7 +16855,7 @@
         <v>65.522800000000004</v>
       </c>
     </row>
-    <row r="227" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
         <v>33</v>
       </c>
@@ -16890,7 +16890,7 @@
         <v>85.823300000000003</v>
       </c>
     </row>
-    <row r="228" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
         <v>33</v>
       </c>
@@ -16925,7 +16925,7 @@
         <v>5.9260999999999999</v>
       </c>
     </row>
-    <row r="229" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
         <v>33</v>
       </c>
@@ -16960,7 +16960,7 @@
         <v>8.5000000000000006E-2</v>
       </c>
     </row>
-    <row r="230" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
         <v>33</v>
       </c>
@@ -16995,7 +16995,7 @@
         <v>65.522800000000004</v>
       </c>
     </row>
-    <row r="231" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
         <v>33</v>
       </c>
@@ -17030,7 +17030,7 @@
         <v>15.885</v>
       </c>
     </row>
-    <row r="232" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
         <v>33</v>
       </c>
@@ -17065,7 +17065,7 @@
         <v>15.885</v>
       </c>
     </row>
-    <row r="233" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
         <v>33</v>
       </c>
@@ -17100,7 +17100,7 @@
         <v>1.7131000000000001</v>
       </c>
     </row>
-    <row r="234" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>33</v>
       </c>
@@ -17135,7 +17135,7 @@
         <v>85.823300000000003</v>
       </c>
     </row>
-    <row r="235" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>33</v>
       </c>
@@ -17170,7 +17170,7 @@
         <v>5.9260999999999999</v>
       </c>
     </row>
-    <row r="236" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
         <v>33</v>
       </c>
@@ -17205,7 +17205,7 @@
         <v>8.5000000000000006E-2</v>
       </c>
     </row>
-    <row r="237" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
         <v>33</v>
       </c>
@@ -17240,7 +17240,7 @@
         <v>65.522800000000004</v>
       </c>
     </row>
-    <row r="238" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
         <v>33</v>
       </c>
@@ -17275,7 +17275,7 @@
         <v>1.7131000000000001</v>
       </c>
     </row>
-    <row r="239" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
         <v>33</v>
       </c>
@@ -17310,7 +17310,7 @@
         <v>85.823300000000003</v>
       </c>
     </row>
-    <row r="240" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
         <v>33</v>
       </c>
@@ -17345,7 +17345,7 @@
         <v>5.9260999999999999</v>
       </c>
     </row>
-    <row r="241" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A241" t="s">
         <v>33</v>
       </c>
@@ -17380,7 +17380,7 @@
         <v>8.5000000000000006E-2</v>
       </c>
     </row>
-    <row r="242" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
         <v>33</v>
       </c>
@@ -17415,7 +17415,7 @@
         <v>65.522800000000004</v>
       </c>
     </row>
-    <row r="243" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
         <v>33</v>
       </c>
@@ -17450,7 +17450,7 @@
         <v>3.3277999999999999</v>
       </c>
     </row>
-    <row r="244" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
         <v>33</v>
       </c>
@@ -17485,7 +17485,7 @@
         <v>3.3277999999999999</v>
       </c>
     </row>
-    <row r="245" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A245" t="s">
         <v>33</v>
       </c>
@@ -17520,7 +17520,7 @@
         <v>1.7131000000000001</v>
       </c>
     </row>
-    <row r="246" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
         <v>33</v>
       </c>
@@ -17555,7 +17555,7 @@
         <v>85.823300000000003</v>
       </c>
     </row>
-    <row r="247" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A247" t="s">
         <v>33</v>
       </c>
@@ -17590,7 +17590,7 @@
         <v>5.9260999999999999</v>
       </c>
     </row>
-    <row r="248" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A248" t="s">
         <v>33</v>
       </c>
@@ -17625,7 +17625,7 @@
         <v>8.5000000000000006E-2</v>
       </c>
     </row>
-    <row r="249" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A249" t="s">
         <v>33</v>
       </c>
@@ -17660,7 +17660,7 @@
         <v>65.522800000000004</v>
       </c>
     </row>
-    <row r="250" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A250" t="s">
         <v>33</v>
       </c>
@@ -17695,7 +17695,7 @@
         <v>1.7131000000000001</v>
       </c>
     </row>
-    <row r="251" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A251" t="s">
         <v>33</v>
       </c>
@@ -17730,7 +17730,7 @@
         <v>18.533899999999999</v>
       </c>
     </row>
-    <row r="252" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
         <v>33</v>
       </c>
@@ -17765,7 +17765,7 @@
         <v>5.9260999999999999</v>
       </c>
     </row>
-    <row r="253" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
         <v>33</v>
       </c>
@@ -17800,7 +17800,7 @@
         <v>2.4902000000000002</v>
       </c>
     </row>
-    <row r="254" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
         <v>33</v>
       </c>
@@ -17835,7 +17835,7 @@
         <v>65.522800000000004</v>
       </c>
     </row>
-    <row r="255" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
         <v>33</v>
       </c>
@@ -17870,7 +17870,7 @@
         <v>0.66279999999999994</v>
       </c>
     </row>
-    <row r="256" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
         <v>33</v>
       </c>
@@ -17905,7 +17905,7 @@
         <v>0.66279999999999994</v>
       </c>
     </row>
-    <row r="257" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
         <v>33</v>
       </c>
@@ -17940,7 +17940,7 @@
         <v>2.2000000000000001E-3</v>
       </c>
     </row>
-    <row r="258" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
         <v>33</v>
       </c>
@@ -17975,7 +17975,7 @@
         <v>18.533899999999999</v>
       </c>
     </row>
-    <row r="259" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
         <v>33</v>
       </c>
@@ -18010,7 +18010,7 @@
         <v>5.9260999999999999</v>
       </c>
     </row>
-    <row r="260" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
         <v>33</v>
       </c>
@@ -18045,7 +18045,7 @@
         <v>2.4902000000000002</v>
       </c>
     </row>
-    <row r="261" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
         <v>33</v>
       </c>
@@ -18080,7 +18080,7 @@
         <v>65.522800000000004</v>
       </c>
     </row>
-    <row r="262" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
         <v>33</v>
       </c>
@@ -18115,7 +18115,7 @@
         <v>2.2000000000000001E-3</v>
       </c>
     </row>
-    <row r="263" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
         <v>33</v>
       </c>
@@ -18150,7 +18150,7 @@
         <v>18.533899999999999</v>
       </c>
     </row>
-    <row r="264" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
         <v>33</v>
       </c>
@@ -18185,7 +18185,7 @@
         <v>5.9260999999999999</v>
       </c>
     </row>
-    <row r="265" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
         <v>33</v>
       </c>
@@ -18220,7 +18220,7 @@
         <v>2.4902000000000002</v>
       </c>
     </row>
-    <row r="266" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
         <v>33</v>
       </c>
@@ -18255,7 +18255,7 @@
         <v>65.522800000000004</v>
       </c>
     </row>
-    <row r="267" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
         <v>33</v>
       </c>
@@ -18290,7 +18290,7 @@
         <v>0.12089999999999999</v>
       </c>
     </row>
-    <row r="268" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
         <v>33</v>
       </c>
@@ -18325,7 +18325,7 @@
         <v>0.12089999999999999</v>
       </c>
     </row>
-    <row r="269" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
         <v>33</v>
       </c>
@@ -18360,7 +18360,7 @@
         <v>2.2000000000000001E-3</v>
       </c>
     </row>
-    <row r="270" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
         <v>33</v>
       </c>
@@ -18395,7 +18395,7 @@
         <v>18.533899999999999</v>
       </c>
     </row>
-    <row r="271" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
         <v>33</v>
       </c>
@@ -18430,7 +18430,7 @@
         <v>5.9260999999999999</v>
       </c>
     </row>
-    <row r="272" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
         <v>33</v>
       </c>
@@ -18465,7 +18465,7 @@
         <v>2.4902000000000002</v>
       </c>
     </row>
-    <row r="273" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A273" t="s">
         <v>33</v>
       </c>
@@ -18500,7 +18500,7 @@
         <v>65.522800000000004</v>
       </c>
     </row>
-    <row r="274" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
         <v>33</v>
       </c>
@@ -18535,7 +18535,7 @@
         <v>2.2000000000000001E-3</v>
       </c>
     </row>
-    <row r="275" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
         <v>33</v>
       </c>
@@ -18570,7 +18570,7 @@
         <v>18.533899999999999</v>
       </c>
     </row>
-    <row r="276" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
         <v>33</v>
       </c>
@@ -18605,7 +18605,7 @@
         <v>2.2000000000000001E-3</v>
       </c>
     </row>
-    <row r="277" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
         <v>33</v>
       </c>
@@ -18640,7 +18640,7 @@
         <v>2.4902000000000002</v>
       </c>
     </row>
-    <row r="278" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
         <v>33</v>
       </c>
@@ -18675,7 +18675,7 @@
         <v>2.2000000000000001E-3</v>
       </c>
     </row>
-    <row r="279" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
         <v>33</v>
       </c>
@@ -18710,7 +18710,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="280" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
         <v>33</v>
       </c>
@@ -18745,7 +18745,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="281" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
         <v>33</v>
       </c>
@@ -18780,7 +18780,7 @@
         <v>2.2000000000000001E-3</v>
       </c>
     </row>
-    <row r="282" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
         <v>33</v>
       </c>
@@ -18815,7 +18815,7 @@
         <v>18.533899999999999</v>
       </c>
     </row>
-    <row r="283" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
         <v>33</v>
       </c>
@@ -18850,7 +18850,7 @@
         <v>2.2000000000000001E-3</v>
       </c>
     </row>
-    <row r="284" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
         <v>33</v>
       </c>
@@ -18885,7 +18885,7 @@
         <v>2.4902000000000002</v>
       </c>
     </row>
-    <row r="285" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
         <v>33</v>
       </c>
@@ -18920,7 +18920,7 @@
         <v>2.2000000000000001E-3</v>
       </c>
     </row>
-    <row r="286" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
         <v>33</v>
       </c>
@@ -18955,7 +18955,7 @@
         <v>2.2000000000000001E-3</v>
       </c>
     </row>
-    <row r="287" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
         <v>23</v>
       </c>
@@ -18990,7 +18990,7 @@
         <v>6.4231999999999996</v>
       </c>
     </row>
-    <row r="288" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
         <v>23</v>
       </c>
@@ -19025,7 +19025,7 @@
         <v>6.4231999999999996</v>
       </c>
     </row>
-    <row r="289" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
         <v>23</v>
       </c>
@@ -19060,7 +19060,7 @@
         <v>93.316599999999994</v>
       </c>
     </row>
-    <row r="290" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A290" t="s">
         <v>23</v>
       </c>
@@ -19095,7 +19095,7 @@
         <v>93.316599999999994</v>
       </c>
     </row>
-    <row r="291" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A291" t="s">
         <v>23</v>
       </c>
@@ -19130,7 +19130,7 @@
         <v>1907.4417000000001</v>
       </c>
     </row>
-    <row r="292" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A292" t="s">
         <v>23</v>
       </c>
@@ -19165,7 +19165,7 @@
         <v>1907.4417000000001</v>
       </c>
     </row>
-    <row r="293" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A293" t="s">
         <v>23</v>
       </c>
@@ -19200,7 +19200,7 @@
         <v>6.4231999999999996</v>
       </c>
     </row>
-    <row r="294" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A294" t="s">
         <v>23</v>
       </c>
@@ -19235,7 +19235,7 @@
         <v>93.316599999999994</v>
       </c>
     </row>
-    <row r="295" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A295" t="s">
         <v>23</v>
       </c>
@@ -19270,7 +19270,7 @@
         <v>5.3855000000000004</v>
       </c>
     </row>
-    <row r="296" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A296" t="s">
         <v>23</v>
       </c>
@@ -19305,7 +19305,7 @@
         <v>5.3855000000000004</v>
       </c>
     </row>
-    <row r="297" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
         <v>23</v>
       </c>
@@ -19340,7 +19340,7 @@
         <v>19.828600000000002</v>
       </c>
     </row>
-    <row r="298" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
         <v>23</v>
       </c>
@@ -19375,7 +19375,7 @@
         <v>19.828600000000002</v>
       </c>
     </row>
-    <row r="299" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A299" t="s">
         <v>23</v>
       </c>
@@ -19410,7 +19410,7 @@
         <v>420.09300000000002</v>
       </c>
     </row>
-    <row r="300" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A300" t="s">
         <v>23</v>
       </c>
@@ -19445,7 +19445,7 @@
         <v>420.09300000000002</v>
       </c>
     </row>
-    <row r="301" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
         <v>23</v>
       </c>
@@ -19480,7 +19480,7 @@
         <v>6.4231999999999996</v>
       </c>
     </row>
-    <row r="302" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A302" t="s">
         <v>23</v>
       </c>
@@ -19515,7 +19515,7 @@
         <v>93.316599999999994</v>
       </c>
     </row>
-    <row r="303" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A303" t="s">
         <v>23</v>
       </c>
@@ -19550,7 +19550,7 @@
         <v>1048.6935000000001</v>
       </c>
     </row>
-    <row r="304" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A304" t="s">
         <v>23</v>
       </c>
@@ -19585,7 +19585,7 @@
         <v>1048.6935000000001</v>
       </c>
     </row>
-    <row r="305" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
         <v>23</v>
       </c>
@@ -19620,7 +19620,7 @@
         <v>80.781099999999995</v>
       </c>
     </row>
-    <row r="306" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
         <v>23</v>
       </c>
@@ -19655,7 +19655,7 @@
         <v>80.781099999999995</v>
       </c>
     </row>
-    <row r="307" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
         <v>23</v>
       </c>
@@ -19690,7 +19690,7 @@
         <v>6.4231999999999996</v>
       </c>
     </row>
-    <row r="308" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A308" t="s">
         <v>23</v>
       </c>
@@ -19725,7 +19725,7 @@
         <v>93.316599999999994</v>
       </c>
     </row>
-    <row r="309" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A309" t="s">
         <v>23</v>
       </c>
@@ -19760,7 +19760,7 @@
         <v>1015.9133</v>
       </c>
     </row>
-    <row r="310" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
         <v>23</v>
       </c>
@@ -19795,7 +19795,7 @@
         <v>1015.9133</v>
       </c>
     </row>
-    <row r="311" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
         <v>23</v>
       </c>
@@ -19830,7 +19830,7 @@
         <v>16.0199</v>
       </c>
     </row>
-    <row r="312" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A312" t="s">
         <v>23</v>
       </c>
@@ -19865,7 +19865,7 @@
         <v>16.0199</v>
       </c>
     </row>
-    <row r="313" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
         <v>23</v>
       </c>
@@ -19900,7 +19900,7 @@
         <v>6.4231999999999996</v>
       </c>
     </row>
-    <row r="314" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
         <v>23</v>
       </c>
@@ -19935,7 +19935,7 @@
         <v>93.316599999999994</v>
       </c>
     </row>
-    <row r="315" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A315" t="s">
         <v>23</v>
       </c>
@@ -19970,7 +19970,7 @@
         <v>19.8659</v>
       </c>
     </row>
-    <row r="316" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A316" t="s">
         <v>23</v>
       </c>
@@ -20005,7 +20005,7 @@
         <v>19.8659</v>
       </c>
     </row>
-    <row r="317" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A317" t="s">
         <v>23</v>
       </c>
@@ -20040,7 +20040,7 @@
         <v>1.06E-2</v>
       </c>
     </row>
-    <row r="318" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A318" t="s">
         <v>23</v>
       </c>
@@ -20075,7 +20075,7 @@
         <v>1.06E-2</v>
       </c>
     </row>
-    <row r="319" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A319" t="s">
         <v>23</v>
       </c>
@@ -20110,7 +20110,7 @@
         <v>3.3250999999999999</v>
       </c>
     </row>
-    <row r="320" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A320" t="s">
         <v>23</v>
       </c>
@@ -20145,7 +20145,7 @@
         <v>3.3250999999999999</v>
       </c>
     </row>
-    <row r="321" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A321" t="s">
         <v>23</v>
       </c>
@@ -20180,7 +20180,7 @@
         <v>19.8659</v>
       </c>
     </row>
-    <row r="322" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A322" t="s">
         <v>23</v>
       </c>
@@ -20215,7 +20215,7 @@
         <v>3.9657</v>
       </c>
     </row>
-    <row r="323" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A323" t="s">
         <v>23</v>
       </c>
@@ -20250,7 +20250,7 @@
         <v>17.7333</v>
       </c>
     </row>
-    <row r="324" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A324" t="s">
         <v>23</v>
       </c>
@@ -20285,7 +20285,7 @@
         <v>17.7333</v>
       </c>
     </row>
-    <row r="325" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A325" t="s">
         <v>23</v>
       </c>
@@ -20320,7 +20320,7 @@
         <v>1.06E-2</v>
       </c>
     </row>
-    <row r="326" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A326" t="s">
         <v>23</v>
       </c>
@@ -20355,7 +20355,7 @@
         <v>1.06E-2</v>
       </c>
     </row>
-    <row r="327" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A327" t="s">
         <v>23</v>
       </c>
@@ -20390,7 +20390,7 @@
         <v>0.59079999999999999</v>
       </c>
     </row>
-    <row r="328" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A328" t="s">
         <v>23</v>
       </c>
@@ -20425,7 +20425,7 @@
         <v>0.59079999999999999</v>
       </c>
     </row>
-    <row r="329" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A329" t="s">
         <v>23</v>
       </c>
@@ -20460,7 +20460,7 @@
         <v>19.8659</v>
       </c>
     </row>
-    <row r="330" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A330" t="s">
         <v>23</v>
       </c>
@@ -20495,7 +20495,7 @@
         <v>3.9657</v>
       </c>
     </row>
-    <row r="331" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A331" t="s">
         <v>23</v>
       </c>
@@ -20530,7 +20530,7 @@
         <v>18.859100000000002</v>
       </c>
     </row>
-    <row r="332" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A332" t="s">
         <v>23</v>
       </c>
@@ -20565,7 +20565,7 @@
         <v>18.859100000000002</v>
       </c>
     </row>
-    <row r="333" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A333" t="s">
         <v>23</v>
       </c>
@@ -20600,7 +20600,7 @@
         <v>1.06E-2</v>
       </c>
     </row>
-    <row r="334" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A334" t="s">
         <v>23</v>
       </c>
@@ -20635,7 +20635,7 @@
         <v>1.06E-2</v>
       </c>
     </row>
-    <row r="335" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A335" t="s">
         <v>23</v>
       </c>
@@ -20670,7 +20670,7 @@
         <v>0.1318</v>
       </c>
     </row>
-    <row r="336" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A336" t="s">
         <v>23</v>
       </c>
@@ -20705,7 +20705,7 @@
         <v>0.1318</v>
       </c>
     </row>
-    <row r="337" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A337" t="s">
         <v>23</v>
       </c>
@@ -20740,7 +20740,7 @@
         <v>19.8659</v>
       </c>
     </row>
-    <row r="338" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A338" t="s">
         <v>23</v>
       </c>
@@ -20775,7 +20775,7 @@
         <v>3.9657</v>
       </c>
     </row>
-    <row r="339" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A339" t="s">
         <v>23</v>
       </c>
@@ -20810,7 +20810,7 @@
         <v>21.3675</v>
       </c>
     </row>
-    <row r="340" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A340" t="s">
         <v>23</v>
       </c>
@@ -20845,7 +20845,7 @@
         <v>21.3675</v>
       </c>
     </row>
-    <row r="341" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A341" t="s">
         <v>23</v>
       </c>
@@ -20880,7 +20880,7 @@
         <v>1.06E-2</v>
       </c>
     </row>
-    <row r="342" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A342" t="s">
         <v>23</v>
       </c>
@@ -20915,7 +20915,7 @@
         <v>1.06E-2</v>
       </c>
     </row>
-    <row r="343" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A343" t="s">
         <v>23</v>
       </c>
@@ -20950,7 +20950,7 @@
         <v>2.8999999999999998E-3</v>
       </c>
     </row>
-    <row r="344" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A344" t="s">
         <v>23</v>
       </c>
@@ -20985,7 +20985,7 @@
         <v>2.8999999999999998E-3</v>
       </c>
     </row>
-    <row r="345" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A345" t="s">
         <v>23</v>
       </c>
@@ -21020,7 +21020,7 @@
         <v>19.8659</v>
       </c>
     </row>
-    <row r="346" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A346" t="s">
         <v>23</v>
       </c>

</xml_diff>